<commit_message>
Added Updated Tables -Lee
</commit_message>
<xml_diff>
--- a/Lee_Ex3A_tables.xlsx
+++ b/Lee_Ex3A_tables.xlsx
@@ -1,19 +1,19 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30430"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://yearuptemp-my.sharepoint.com/personal/ilee_my_yearupunited_org/Documents/Documents/DATA_Labs/W2_Workshop/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="89" documentId="11_E60897F41BE170836B02CE998F75CCDC64E183C8" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{6F2C300F-7EE8-4F25-8913-658CFB5406DE}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{F1C019C2-B7D8-4D88-9558-B9293B7383EA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-96" yWindow="0" windowWidth="11712" windowHeight="13776" firstSheet="3" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="23040" windowHeight="13680" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="ClLIENTS" sheetId="1" r:id="rId1"/>
+    <sheet name="CLIENTS" sheetId="1" r:id="rId1"/>
     <sheet name="DOGS" sheetId="2" r:id="rId2"/>
     <sheet name="WALKERS" sheetId="3" r:id="rId3"/>
     <sheet name="SERVICE_TYPES" sheetId="4" r:id="rId4"/>
@@ -43,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="29" uniqueCount="25">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="230" uniqueCount="162">
   <si>
     <t>client_name</t>
   </si>
@@ -118,16 +118,446 @@
   </si>
   <si>
     <t>walk_notes</t>
+  </si>
+  <si>
+    <t>C01</t>
+  </si>
+  <si>
+    <t>527 Benedict St.</t>
+  </si>
+  <si>
+    <t>Pennsauken</t>
+  </si>
+  <si>
+    <t>NJ</t>
+  </si>
+  <si>
+    <t>D01</t>
+  </si>
+  <si>
+    <t>Dawn</t>
+  </si>
+  <si>
+    <t>Syberian Husky</t>
+  </si>
+  <si>
+    <t>gets distracted by squirrels, allergic to cotton candy</t>
+  </si>
+  <si>
+    <t>W01</t>
+  </si>
+  <si>
+    <t>Johnny</t>
+  </si>
+  <si>
+    <t>johnny4dogs@zmail.com</t>
+  </si>
+  <si>
+    <t>SC01</t>
+  </si>
+  <si>
+    <t>30 min walk</t>
+  </si>
+  <si>
+    <t>Henry Wilson</t>
+  </si>
+  <si>
+    <t>Wilson.h@zmail.com</t>
+  </si>
+  <si>
+    <t>C02</t>
+  </si>
+  <si>
+    <t>C03</t>
+  </si>
+  <si>
+    <t>C04</t>
+  </si>
+  <si>
+    <t>C05</t>
+  </si>
+  <si>
+    <t>C06</t>
+  </si>
+  <si>
+    <t>C07</t>
+  </si>
+  <si>
+    <t>C08</t>
+  </si>
+  <si>
+    <t>Maria Santos</t>
+  </si>
+  <si>
+    <t>Derek Park</t>
+  </si>
+  <si>
+    <t>Priya Nair</t>
+  </si>
+  <si>
+    <t>Tom Reilly</t>
+  </si>
+  <si>
+    <t>Aisha Johnson</t>
+  </si>
+  <si>
+    <t>Greg Alvarez</t>
+  </si>
+  <si>
+    <t>Hannah Cole</t>
+  </si>
+  <si>
+    <t>maria.santos@zmail.com</t>
+  </si>
+  <si>
+    <t>priya.nair@zmail.com</t>
+  </si>
+  <si>
+    <t>dpark@zmail.com</t>
+  </si>
+  <si>
+    <t>treilly@zmail.com</t>
+  </si>
+  <si>
+    <t>galvarez@zmail.com</t>
+  </si>
+  <si>
+    <t>aisha.j@zmail.com</t>
+  </si>
+  <si>
+    <t>hcole@zmail.com</t>
+  </si>
+  <si>
+    <t>14 Elm Ave.</t>
+  </si>
+  <si>
+    <t>301 Collings Rd.</t>
+  </si>
+  <si>
+    <t>88 Kings Hwy.</t>
+  </si>
+  <si>
+    <t>42 Maple Ln.</t>
+  </si>
+  <si>
+    <t>19 Chestnut St.</t>
+  </si>
+  <si>
+    <t>655 Rt. 73 N.</t>
+  </si>
+  <si>
+    <t>230 Park Dr.</t>
+  </si>
+  <si>
+    <t>Haddonfield</t>
+  </si>
+  <si>
+    <t>Collingswood</t>
+  </si>
+  <si>
+    <t>Cherry Hill</t>
+  </si>
+  <si>
+    <t>Voorhees</t>
+  </si>
+  <si>
+    <t>Moorestown</t>
+  </si>
+  <si>
+    <t>Marlton</t>
+  </si>
+  <si>
+    <t>08110</t>
+  </si>
+  <si>
+    <t>08033</t>
+  </si>
+  <si>
+    <t>08108</t>
+  </si>
+  <si>
+    <t>08002</t>
+  </si>
+  <si>
+    <t>08043</t>
+  </si>
+  <si>
+    <t>08057</t>
+  </si>
+  <si>
+    <t>08053</t>
+  </si>
+  <si>
+    <t>D02</t>
+  </si>
+  <si>
+    <t>D03</t>
+  </si>
+  <si>
+    <t>D04</t>
+  </si>
+  <si>
+    <t>D05</t>
+  </si>
+  <si>
+    <t>D06</t>
+  </si>
+  <si>
+    <t>D07</t>
+  </si>
+  <si>
+    <t>D08</t>
+  </si>
+  <si>
+    <t>D09</t>
+  </si>
+  <si>
+    <t>D10</t>
+  </si>
+  <si>
+    <t>Biscuit</t>
+  </si>
+  <si>
+    <t>Luna</t>
+  </si>
+  <si>
+    <t>Max</t>
+  </si>
+  <si>
+    <t>Bella</t>
+  </si>
+  <si>
+    <t>Rocky</t>
+  </si>
+  <si>
+    <t>Daisy</t>
+  </si>
+  <si>
+    <t>Cooper</t>
+  </si>
+  <si>
+    <t>Pepper</t>
+  </si>
+  <si>
+    <t>Milo</t>
+  </si>
+  <si>
+    <t>Beagle</t>
+  </si>
+  <si>
+    <t>Labrador Retriever</t>
+  </si>
+  <si>
+    <t>German Shepherd</t>
+  </si>
+  <si>
+    <t>Golden Retriever</t>
+  </si>
+  <si>
+    <t>Boxer</t>
+  </si>
+  <si>
+    <t>Dachshund</t>
+  </si>
+  <si>
+    <t>Border Collie</t>
+  </si>
+  <si>
+    <t>Chihuahua</t>
+  </si>
+  <si>
+    <t>Goldendoodle</t>
+  </si>
+  <si>
+    <t>follows his nose, Loves treats</t>
+  </si>
+  <si>
+    <t>very friendly, pulls at start of walk</t>
+  </si>
+  <si>
+    <t>barks at skateboards and bikes</t>
+  </si>
+  <si>
+    <t>loves water, stop at puddles</t>
+  </si>
+  <si>
+    <t>strong puller, use harness</t>
+  </si>
+  <si>
+    <t>short walks only, back issues</t>
+  </si>
+  <si>
+    <t>herds other dogs, needs lots of exercise</t>
+  </si>
+  <si>
+    <t>scared of large dogs, carry across busy streets</t>
+  </si>
+  <si>
+    <t>allergic to chicken treats</t>
+  </si>
+  <si>
+    <t>Sofia</t>
+  </si>
+  <si>
+    <t>Marcus</t>
+  </si>
+  <si>
+    <t>Tess</t>
+  </si>
+  <si>
+    <t>sofia.walks@zmail.com</t>
+  </si>
+  <si>
+    <t>marcus.pawpatrol@zmail.com</t>
+  </si>
+  <si>
+    <t>tess4tails@zmail.com</t>
+  </si>
+  <si>
+    <t>SC02</t>
+  </si>
+  <si>
+    <t>SC03</t>
+  </si>
+  <si>
+    <t>SC04</t>
+  </si>
+  <si>
+    <t>SC05</t>
+  </si>
+  <si>
+    <t>45 min walk</t>
+  </si>
+  <si>
+    <t>60 min walk</t>
+  </si>
+  <si>
+    <t>Puppy visit</t>
+  </si>
+  <si>
+    <t>Group Adventure</t>
+  </si>
+  <si>
+    <t>W02</t>
+  </si>
+  <si>
+    <t>W03</t>
+  </si>
+  <si>
+    <t>W04</t>
+  </si>
+  <si>
+    <t>WK01</t>
+  </si>
+  <si>
+    <t>WK02</t>
+  </si>
+  <si>
+    <t>WK03</t>
+  </si>
+  <si>
+    <t>WK04</t>
+  </si>
+  <si>
+    <t>WK05</t>
+  </si>
+  <si>
+    <t>WK06</t>
+  </si>
+  <si>
+    <t>WK07</t>
+  </si>
+  <si>
+    <t>WK08</t>
+  </si>
+  <si>
+    <t>WK09</t>
+  </si>
+  <si>
+    <t>WK10</t>
+  </si>
+  <si>
+    <t>WK11</t>
+  </si>
+  <si>
+    <t>WK12</t>
+  </si>
+  <si>
+    <t>WK13</t>
+  </si>
+  <si>
+    <t>WK14</t>
+  </si>
+  <si>
+    <t>WK15</t>
+  </si>
+  <si>
+    <t>Chased a squirrel twice, recovered fast</t>
+  </si>
+  <si>
+    <t>Great leash maners today</t>
+  </si>
+  <si>
+    <t>Short loop, took breaks often</t>
+  </si>
+  <si>
+    <t>Barked at a cyclist, redirected with treat</t>
+  </si>
+  <si>
+    <t>Carried across Kings Hwy.</t>
+  </si>
+  <si>
+    <t>Herded two beagles at dog park</t>
+  </si>
+  <si>
+    <t>Pulled hard at start, harness helped</t>
+  </si>
+  <si>
+    <t>Met a friendly poodle, no issues</t>
+  </si>
+  <si>
+    <t>Skipped treats, avioded chicken</t>
+  </si>
+  <si>
+    <t>Calm and relaxed</t>
+  </si>
+  <si>
+    <t>Led the group on the trail</t>
+  </si>
+  <si>
+    <t>Fast walker, covered extra ground</t>
+  </si>
+  <si>
+    <t>Nervous near school crossing</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <numFmts count="3">
+    <numFmt numFmtId="164" formatCode="0.00;[Red]0.00"/>
+    <numFmt numFmtId="165" formatCode="yyyy\-mm\-dd;@"/>
+    <numFmt numFmtId="166" formatCode="#,##0.00;[Red]#,##0.00"/>
+  </numFmts>
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="10"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="8"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -162,18 +592,27 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1"/>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="18" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="21" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -486,13 +925,15 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:H1"/>
+  <dimension ref="A1:H9"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="9.88671875" customWidth="1"/>
     <col min="2" max="2" width="12.77734375" customWidth="1"/>
-    <col min="3" max="3" width="16.88671875" customWidth="1"/>
-    <col min="4" max="4" width="12.5546875" customWidth="1"/>
+    <col min="3" max="3" width="22" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="12.77734375" customWidth="1"/>
+    <col min="5" max="5" width="13.77734375" customWidth="1"/>
+    <col min="6" max="6" width="11.88671875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.3">
@@ -521,19 +962,238 @@
         <v>7</v>
       </c>
     </row>
+    <row r="2" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
+        <v>25</v>
+      </c>
+      <c r="B2" t="s">
+        <v>38</v>
+      </c>
+      <c r="C2" s="4" t="s">
+        <v>39</v>
+      </c>
+      <c r="D2" s="5">
+        <v>8565550101</v>
+      </c>
+      <c r="E2" t="s">
+        <v>26</v>
+      </c>
+      <c r="F2" t="s">
+        <v>27</v>
+      </c>
+      <c r="G2" t="s">
+        <v>28</v>
+      </c>
+      <c r="H2" s="5" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
+        <v>40</v>
+      </c>
+      <c r="B3" t="s">
+        <v>47</v>
+      </c>
+      <c r="C3" s="4" t="s">
+        <v>54</v>
+      </c>
+      <c r="D3" s="5">
+        <v>8565550102</v>
+      </c>
+      <c r="E3" t="s">
+        <v>61</v>
+      </c>
+      <c r="F3" t="s">
+        <v>68</v>
+      </c>
+      <c r="G3" t="s">
+        <v>28</v>
+      </c>
+      <c r="H3" s="5" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
+        <v>41</v>
+      </c>
+      <c r="B4" t="s">
+        <v>48</v>
+      </c>
+      <c r="C4" s="4" t="s">
+        <v>56</v>
+      </c>
+      <c r="D4" s="5">
+        <v>8565550103</v>
+      </c>
+      <c r="E4" t="s">
+        <v>62</v>
+      </c>
+      <c r="F4" t="s">
+        <v>69</v>
+      </c>
+      <c r="G4" t="s">
+        <v>28</v>
+      </c>
+      <c r="H4" s="5" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A5" t="s">
+        <v>42</v>
+      </c>
+      <c r="B5" t="s">
+        <v>49</v>
+      </c>
+      <c r="C5" s="4" t="s">
+        <v>55</v>
+      </c>
+      <c r="D5" s="5">
+        <v>8565550104</v>
+      </c>
+      <c r="E5" t="s">
+        <v>63</v>
+      </c>
+      <c r="F5" t="s">
+        <v>70</v>
+      </c>
+      <c r="G5" t="s">
+        <v>28</v>
+      </c>
+      <c r="H5" s="5" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A6" t="s">
+        <v>43</v>
+      </c>
+      <c r="B6" t="s">
+        <v>50</v>
+      </c>
+      <c r="C6" s="4" t="s">
+        <v>57</v>
+      </c>
+      <c r="D6" s="5">
+        <v>8565550105</v>
+      </c>
+      <c r="E6" t="s">
+        <v>64</v>
+      </c>
+      <c r="F6" t="s">
+        <v>71</v>
+      </c>
+      <c r="G6" t="s">
+        <v>28</v>
+      </c>
+      <c r="H6" s="5" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A7" t="s">
+        <v>44</v>
+      </c>
+      <c r="B7" t="s">
+        <v>51</v>
+      </c>
+      <c r="C7" s="4" t="s">
+        <v>59</v>
+      </c>
+      <c r="D7" s="5">
+        <v>8565550106</v>
+      </c>
+      <c r="E7" t="s">
+        <v>65</v>
+      </c>
+      <c r="F7" t="s">
+        <v>72</v>
+      </c>
+      <c r="G7" t="s">
+        <v>28</v>
+      </c>
+      <c r="H7" s="5" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A8" t="s">
+        <v>45</v>
+      </c>
+      <c r="B8" t="s">
+        <v>52</v>
+      </c>
+      <c r="C8" s="4" t="s">
+        <v>58</v>
+      </c>
+      <c r="D8" s="5">
+        <v>856555017</v>
+      </c>
+      <c r="E8" t="s">
+        <v>66</v>
+      </c>
+      <c r="F8" t="s">
+        <v>73</v>
+      </c>
+      <c r="G8" t="s">
+        <v>28</v>
+      </c>
+      <c r="H8" s="5" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A9" t="s">
+        <v>46</v>
+      </c>
+      <c r="B9" t="s">
+        <v>53</v>
+      </c>
+      <c r="C9" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="D9" s="5">
+        <v>8565550108</v>
+      </c>
+      <c r="E9" t="s">
+        <v>67</v>
+      </c>
+      <c r="F9" t="s">
+        <v>27</v>
+      </c>
+      <c r="G9" t="s">
+        <v>28</v>
+      </c>
+      <c r="H9" s="5" t="s">
+        <v>74</v>
+      </c>
+    </row>
   </sheetData>
+  <hyperlinks>
+    <hyperlink ref="C2" r:id="rId1" xr:uid="{A273F5A3-CF7B-4CC1-8111-88A0B07E92A7}"/>
+    <hyperlink ref="C3" r:id="rId2" xr:uid="{27EF0F45-5808-4C07-9C8F-462A0FAB2423}"/>
+    <hyperlink ref="C4" r:id="rId3" xr:uid="{68B76659-34EE-4250-B6DD-0E350E5AD0C4}"/>
+    <hyperlink ref="C5" r:id="rId4" xr:uid="{905B75AF-E0E3-4396-B0FF-28B211E9F831}"/>
+    <hyperlink ref="C6" r:id="rId5" xr:uid="{04C0B059-646E-443F-A094-5BF92BAC1DA0}"/>
+    <hyperlink ref="C8" r:id="rId6" xr:uid="{20D58DEE-9F4A-4AEE-AE26-079358F96922}"/>
+    <hyperlink ref="C7" r:id="rId7" xr:uid="{F6998E62-006D-4439-B64E-BE27463492F0}"/>
+    <hyperlink ref="C9" r:id="rId8" xr:uid="{643F0784-CDEA-47E3-B920-51085571E3E0}"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId1"/>
+  <pageSetup orientation="portrait" r:id="rId9"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3E1F5C9C-2387-4CD9-9A93-4D162C1EA1F7}">
-  <dimension ref="A1:E1"/>
+  <dimension ref="A1:E11"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="2" width="10.5546875" customWidth="1"/>
-    <col min="4" max="4" width="12.33203125" customWidth="1"/>
+    <col min="3" max="3" width="16.33203125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="43.33203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.3">
@@ -553,17 +1213,189 @@
         <v>1</v>
       </c>
     </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
+        <v>29</v>
+      </c>
+      <c r="B2" t="s">
+        <v>30</v>
+      </c>
+      <c r="C2" t="s">
+        <v>31</v>
+      </c>
+      <c r="D2" t="s">
+        <v>32</v>
+      </c>
+      <c r="E2" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
+        <v>81</v>
+      </c>
+      <c r="B3" t="s">
+        <v>90</v>
+      </c>
+      <c r="C3" t="s">
+        <v>99</v>
+      </c>
+      <c r="D3" t="s">
+        <v>108</v>
+      </c>
+      <c r="E3" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
+        <v>82</v>
+      </c>
+      <c r="B4" t="s">
+        <v>91</v>
+      </c>
+      <c r="C4" t="s">
+        <v>100</v>
+      </c>
+      <c r="D4" t="s">
+        <v>109</v>
+      </c>
+      <c r="E4" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A5" t="s">
+        <v>83</v>
+      </c>
+      <c r="B5" t="s">
+        <v>92</v>
+      </c>
+      <c r="C5" t="s">
+        <v>101</v>
+      </c>
+      <c r="D5" t="s">
+        <v>110</v>
+      </c>
+      <c r="E5" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A6" t="s">
+        <v>84</v>
+      </c>
+      <c r="B6" t="s">
+        <v>93</v>
+      </c>
+      <c r="C6" t="s">
+        <v>102</v>
+      </c>
+      <c r="D6" t="s">
+        <v>111</v>
+      </c>
+      <c r="E6" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A7" t="s">
+        <v>85</v>
+      </c>
+      <c r="B7" t="s">
+        <v>94</v>
+      </c>
+      <c r="C7" t="s">
+        <v>103</v>
+      </c>
+      <c r="D7" t="s">
+        <v>112</v>
+      </c>
+      <c r="E7" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A8" t="s">
+        <v>86</v>
+      </c>
+      <c r="B8" t="s">
+        <v>95</v>
+      </c>
+      <c r="C8" t="s">
+        <v>104</v>
+      </c>
+      <c r="D8" t="s">
+        <v>113</v>
+      </c>
+      <c r="E8" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A9" t="s">
+        <v>87</v>
+      </c>
+      <c r="B9" t="s">
+        <v>96</v>
+      </c>
+      <c r="C9" t="s">
+        <v>105</v>
+      </c>
+      <c r="D9" t="s">
+        <v>114</v>
+      </c>
+      <c r="E9" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A10" t="s">
+        <v>88</v>
+      </c>
+      <c r="B10" t="s">
+        <v>97</v>
+      </c>
+      <c r="C10" t="s">
+        <v>106</v>
+      </c>
+      <c r="D10" t="s">
+        <v>115</v>
+      </c>
+      <c r="E10" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A11" t="s">
+        <v>89</v>
+      </c>
+      <c r="B11" t="s">
+        <v>98</v>
+      </c>
+      <c r="C11" t="s">
+        <v>107</v>
+      </c>
+      <c r="D11" t="s">
+        <v>116</v>
+      </c>
+      <c r="E11" t="s">
+        <v>45</v>
+      </c>
+    </row>
   </sheetData>
+  <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{11E652A4-AED7-4294-A0B0-69E5D7EB0103}">
-  <dimension ref="A1:D1"/>
+  <dimension ref="A1:D5"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="2" max="3" width="12.6640625" customWidth="1"/>
+    <col min="2" max="2" width="12.6640625" customWidth="1"/>
+    <col min="3" max="3" width="26.33203125" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="12.5546875" customWidth="1"/>
   </cols>
   <sheetData>
@@ -581,17 +1413,81 @@
         <v>15</v>
       </c>
     </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
+        <v>33</v>
+      </c>
+      <c r="B2" t="s">
+        <v>34</v>
+      </c>
+      <c r="C2" s="4" t="s">
+        <v>35</v>
+      </c>
+      <c r="D2">
+        <v>8563330201</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
+        <v>131</v>
+      </c>
+      <c r="B3" t="s">
+        <v>117</v>
+      </c>
+      <c r="C3" s="4" t="s">
+        <v>120</v>
+      </c>
+      <c r="D3">
+        <v>8563330202</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
+        <v>132</v>
+      </c>
+      <c r="B4" t="s">
+        <v>118</v>
+      </c>
+      <c r="C4" s="4" t="s">
+        <v>121</v>
+      </c>
+      <c r="D4">
+        <v>8563330203</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A5" t="s">
+        <v>133</v>
+      </c>
+      <c r="B5" t="s">
+        <v>119</v>
+      </c>
+      <c r="C5" s="4" t="s">
+        <v>122</v>
+      </c>
+      <c r="D5">
+        <v>8563330204</v>
+      </c>
+    </row>
   </sheetData>
+  <phoneticPr fontId="2" type="noConversion"/>
+  <hyperlinks>
+    <hyperlink ref="C2" r:id="rId1" xr:uid="{C05D261C-7780-4790-AFE7-EB7D6C5C55DF}"/>
+    <hyperlink ref="C3" r:id="rId2" xr:uid="{6B113278-D9B9-4D1C-83D0-C975FC957EDD}"/>
+    <hyperlink ref="C4" r:id="rId3" xr:uid="{7B1501F8-182F-423E-9833-01FBEFCF96F9}"/>
+    <hyperlink ref="C5" r:id="rId4" xr:uid="{D2C9D426-5664-40F6-90D1-D4FA1C8DBFCF}"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{40C08D94-00E3-42E6-B295-DCBBFCF04AA3}">
-  <dimension ref="A1:D1"/>
+  <dimension ref="A1:D6"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="2" width="12.5546875" customWidth="1"/>
+    <col min="1" max="1" width="12.5546875" customWidth="1"/>
+    <col min="2" max="2" width="14.88671875" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="14.33203125" customWidth="1"/>
     <col min="4" max="4" width="13.88671875" customWidth="1"/>
   </cols>
@@ -610,20 +1506,91 @@
         <v>19</v>
       </c>
     </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
+        <v>36</v>
+      </c>
+      <c r="B2" t="s">
+        <v>37</v>
+      </c>
+      <c r="C2">
+        <v>30</v>
+      </c>
+      <c r="D2" s="6">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
+        <v>123</v>
+      </c>
+      <c r="B3" t="s">
+        <v>127</v>
+      </c>
+      <c r="C3">
+        <v>45</v>
+      </c>
+      <c r="D3" s="6">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
+        <v>124</v>
+      </c>
+      <c r="B4" t="s">
+        <v>128</v>
+      </c>
+      <c r="C4">
+        <v>60</v>
+      </c>
+      <c r="D4" s="6">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A5" t="s">
+        <v>125</v>
+      </c>
+      <c r="B5" t="s">
+        <v>129</v>
+      </c>
+      <c r="C5">
+        <v>20</v>
+      </c>
+      <c r="D5" s="6">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A6" t="s">
+        <v>126</v>
+      </c>
+      <c r="B6" t="s">
+        <v>130</v>
+      </c>
+      <c r="C6">
+        <v>90</v>
+      </c>
+      <c r="D6" s="6">
+        <v>45</v>
+      </c>
+    </row>
   </sheetData>
+  <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F98B01E6-2367-4C94-86A5-80C2DE892151}">
-  <dimension ref="A1:H1"/>
+  <dimension ref="A1:H16"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="2" max="2" width="9.88671875" customWidth="1"/>
-    <col min="3" max="3" width="10" customWidth="1"/>
+    <col min="2" max="2" width="10.5546875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="9.44140625" style="8" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="15.77734375" customWidth="1"/>
-    <col min="5" max="5" width="10.5546875" customWidth="1"/>
+    <col min="5" max="5" width="34" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="10.88671875" customWidth="1"/>
   </cols>
   <sheetData>
@@ -634,7 +1601,7 @@
       <c r="B1" t="s">
         <v>21</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="10" t="s">
         <v>22</v>
       </c>
       <c r="D1" t="s">
@@ -653,7 +1620,392 @@
         <v>16</v>
       </c>
     </row>
+    <row r="2" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
+        <v>134</v>
+      </c>
+      <c r="B2" s="7">
+        <v>46300</v>
+      </c>
+      <c r="C2" s="8">
+        <v>0.33333333333333331</v>
+      </c>
+      <c r="D2" s="9">
+        <v>20</v>
+      </c>
+      <c r="E2" t="s">
+        <v>149</v>
+      </c>
+      <c r="F2" t="s">
+        <v>29</v>
+      </c>
+      <c r="G2" t="s">
+        <v>33</v>
+      </c>
+      <c r="H2" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
+        <v>135</v>
+      </c>
+      <c r="B3" s="7">
+        <v>46300</v>
+      </c>
+      <c r="C3" s="8">
+        <v>0.39583333333333331</v>
+      </c>
+      <c r="D3" s="9">
+        <v>35</v>
+      </c>
+      <c r="E3" t="s">
+        <v>150</v>
+      </c>
+      <c r="F3" t="s">
+        <v>84</v>
+      </c>
+      <c r="G3" t="s">
+        <v>131</v>
+      </c>
+      <c r="H3" t="s">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
+        <v>136</v>
+      </c>
+      <c r="B4" s="7">
+        <v>46301</v>
+      </c>
+      <c r="C4" s="8">
+        <v>0.5</v>
+      </c>
+      <c r="D4" s="9">
+        <v>20</v>
+      </c>
+      <c r="E4" t="s">
+        <v>151</v>
+      </c>
+      <c r="F4" t="s">
+        <v>86</v>
+      </c>
+      <c r="G4" t="s">
+        <v>132</v>
+      </c>
+      <c r="H4" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A5" t="s">
+        <v>137</v>
+      </c>
+      <c r="B5" s="7">
+        <v>46302</v>
+      </c>
+      <c r="C5" s="8">
+        <v>0.6875</v>
+      </c>
+      <c r="D5" s="9">
+        <v>27</v>
+      </c>
+      <c r="E5" t="s">
+        <v>152</v>
+      </c>
+      <c r="F5" t="s">
+        <v>83</v>
+      </c>
+      <c r="G5" t="s">
+        <v>33</v>
+      </c>
+      <c r="H5" t="s">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A6" t="s">
+        <v>138</v>
+      </c>
+      <c r="B6" s="7">
+        <v>46303</v>
+      </c>
+      <c r="C6" s="8">
+        <v>0.82291666666666663</v>
+      </c>
+      <c r="D6" s="9">
+        <v>35</v>
+      </c>
+      <c r="E6" t="s">
+        <v>153</v>
+      </c>
+      <c r="F6" t="s">
+        <v>84</v>
+      </c>
+      <c r="G6" t="s">
+        <v>133</v>
+      </c>
+      <c r="H6" t="s">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A7" t="s">
+        <v>139</v>
+      </c>
+      <c r="B7" s="7">
+        <v>46304</v>
+      </c>
+      <c r="C7" s="8">
+        <v>0.42708333333333331</v>
+      </c>
+      <c r="D7" s="9">
+        <v>15</v>
+      </c>
+      <c r="E7" t="s">
+        <v>154</v>
+      </c>
+      <c r="F7" t="s">
+        <v>88</v>
+      </c>
+      <c r="G7" t="s">
+        <v>131</v>
+      </c>
+      <c r="H7" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A8" t="s">
+        <v>140</v>
+      </c>
+      <c r="B8" s="7">
+        <v>46305</v>
+      </c>
+      <c r="C8" s="8">
+        <v>0.58333333333333337</v>
+      </c>
+      <c r="D8" s="9">
+        <v>45</v>
+      </c>
+      <c r="E8" t="s">
+        <v>155</v>
+      </c>
+      <c r="F8" t="s">
+        <v>87</v>
+      </c>
+      <c r="G8" t="s">
+        <v>132</v>
+      </c>
+      <c r="H8" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A9" t="s">
+        <v>141</v>
+      </c>
+      <c r="B9" s="7">
+        <v>46306</v>
+      </c>
+      <c r="C9" s="8">
+        <v>0.35416666666666669</v>
+      </c>
+      <c r="D9" s="9">
+        <v>27</v>
+      </c>
+      <c r="F9" t="s">
+        <v>85</v>
+      </c>
+      <c r="G9" t="s">
+        <v>33</v>
+      </c>
+      <c r="H9" t="s">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="10" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A10" t="s">
+        <v>142</v>
+      </c>
+      <c r="B10" s="7">
+        <v>46307</v>
+      </c>
+      <c r="C10" s="8">
+        <v>0.45833333333333331</v>
+      </c>
+      <c r="D10" s="9">
+        <v>20</v>
+      </c>
+      <c r="E10" t="s">
+        <v>156</v>
+      </c>
+      <c r="F10" t="s">
+        <v>81</v>
+      </c>
+      <c r="G10" t="s">
+        <v>133</v>
+      </c>
+      <c r="H10" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="11" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A11" t="s">
+        <v>143</v>
+      </c>
+      <c r="B11" s="7">
+        <v>46308</v>
+      </c>
+      <c r="C11" s="8">
+        <v>0.55208333333333337</v>
+      </c>
+      <c r="D11" s="9">
+        <v>27</v>
+      </c>
+      <c r="E11" t="s">
+        <v>157</v>
+      </c>
+      <c r="F11" t="s">
+        <v>82</v>
+      </c>
+      <c r="G11" t="s">
+        <v>131</v>
+      </c>
+      <c r="H11" t="s">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="12" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A12" t="s">
+        <v>144</v>
+      </c>
+      <c r="B12" s="7">
+        <v>46309</v>
+      </c>
+      <c r="C12" s="8">
+        <v>0.375</v>
+      </c>
+      <c r="D12" s="9">
+        <v>35</v>
+      </c>
+      <c r="E12" t="s">
+        <v>158</v>
+      </c>
+      <c r="F12" t="s">
+        <v>89</v>
+      </c>
+      <c r="G12" t="s">
+        <v>132</v>
+      </c>
+      <c r="H12" t="s">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="13" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A13" t="s">
+        <v>145</v>
+      </c>
+      <c r="B13" s="7">
+        <v>46310</v>
+      </c>
+      <c r="C13" s="8">
+        <v>0.70833333333333337</v>
+      </c>
+      <c r="D13" s="9">
+        <v>20</v>
+      </c>
+      <c r="E13" t="s">
+        <v>159</v>
+      </c>
+      <c r="F13" t="s">
+        <v>29</v>
+      </c>
+      <c r="G13" t="s">
+        <v>33</v>
+      </c>
+      <c r="H13" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="14" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A14" t="s">
+        <v>146</v>
+      </c>
+      <c r="B14" s="7">
+        <v>46311</v>
+      </c>
+      <c r="C14" s="8">
+        <v>0.84375</v>
+      </c>
+      <c r="D14" s="9">
+        <v>45</v>
+      </c>
+      <c r="E14" t="s">
+        <v>160</v>
+      </c>
+      <c r="F14" t="s">
+        <v>87</v>
+      </c>
+      <c r="G14" t="s">
+        <v>133</v>
+      </c>
+      <c r="H14" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="15" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A15" t="s">
+        <v>147</v>
+      </c>
+      <c r="B15" s="7">
+        <v>46312</v>
+      </c>
+      <c r="C15" s="8">
+        <v>0.52083333333333337</v>
+      </c>
+      <c r="D15" s="9">
+        <v>35</v>
+      </c>
+      <c r="E15" t="s">
+        <v>161</v>
+      </c>
+      <c r="F15" t="s">
+        <v>82</v>
+      </c>
+      <c r="G15" t="s">
+        <v>131</v>
+      </c>
+      <c r="H15" t="s">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="16" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A16" t="s">
+        <v>148</v>
+      </c>
+      <c r="B16" s="7">
+        <v>46313</v>
+      </c>
+      <c r="C16" s="8">
+        <v>0.65625</v>
+      </c>
+      <c r="D16" s="9">
+        <v>15</v>
+      </c>
+      <c r="F16" t="s">
+        <v>88</v>
+      </c>
+      <c r="G16" t="s">
+        <v>132</v>
+      </c>
+      <c r="H16" t="s">
+        <v>125</v>
+      </c>
+    </row>
   </sheetData>
+  <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>